<commit_message>
changed the code to only 3 tabs in excel file report
</commit_message>
<xml_diff>
--- a/2.12.1.345_Test Status Report.xlsx
+++ b/2.12.1.345_Test Status Report.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Online Runs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Online Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curves Runs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curves Results" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curve Runs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary Results" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,19 +627,6 @@
       </c>
       <c r="C15" t="n">
         <v>0.059</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Run 15 - Magnum_380_run_6_5mph_1</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.021</v>
       </c>
     </row>
   </sheetData>
@@ -654,149 +640,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RUN #</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>PEAKS AVG (m)</t>
+          <t>MAXABSIMPXTE (m)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>STATUS - PEAKS AVG</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ABS AVG (m)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS ABS AVG</t>
+          <t>AVGABSIMPXTE (m)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>run 1</t>
+          <t>Run 15 - Magnum_380_run_6_5mph_1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.04033333333333333</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
+        <v>0.081</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.021</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>run 2</t>
+          <t>Run 16 - Magnum_380_run_6_5mph_2</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07333333333333333</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.02066666666666667</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
+        <v>0.062</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>run 3</t>
+          <t>Run 17 - Magnum_380_run_6_5mph_3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.08733333333333333</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
+        <v>0.051</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.015</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>run 4</t>
+          <t>Run 18 - Magnum_380_run_7_5mph_1</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.02833333333333333</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
+        <v>0.097</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>run 5</t>
+          <t>Run 19 - Magnum_380_run_7_5mph_2</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0.04133333333333333</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
+        <v>0.094</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.029</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Run 20 - Magnum_380_run_7_5mph_3</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.027</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Run 21 - Magnum_380_run_8_8mph_1</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.049</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Run 22 - Magnum_380_run_8_8mph_2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.077</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Run 23 - Magnum_380_run_8_8mph_3</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.066</v>
       </c>
     </row>
   </sheetData>
@@ -810,248 +788,215 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>Run</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>MAXABSIMPXTE (m)</t>
+          <t>PEAKS AVG (m)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>AVGABSIMPXTE (m)</t>
+          <t>STATUS - PEAKS AVG</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ABS AVG (m)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS ABS AVG</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run 16 - Magnum_380_run_6_5mph_2</t>
+          <t>run 1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.017</v>
+        <v>0.036</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Run 17 - Magnum_380_run_6_5mph_3</t>
+          <t>run 2</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.051</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.015</v>
+        <v>0.04699999999999999</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.01566666666666667</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Run 18 - Magnum_380_run_7_5mph_1</t>
+          <t>run 3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="C4" t="n">
+        <v>0.09366666666666668</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>0.03</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Run 19 - Magnum_380_run_7_5mph_2</t>
+          <t>run 4</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.029</v>
+        <v>0.09066666666666667</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.03066666666666666</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Run 20 - Magnum_380_run_7_5mph_3</t>
+          <t>run 5</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.092</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.027</v>
+        <v>0.1406666666666667</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.04433333333333334</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Run 21 - Magnum_380_run_8_8mph_1</t>
+          <t>run 6</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.158</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.049</v>
+        <v>0.06466666666666666</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.01766666666666667</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Run 22 - Magnum_380_run_8_8mph_2</t>
+          <t>run 7</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.251</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.077</v>
+        <v>0.09433333333333334</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.02866666666666666</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Run 23 - Magnum_380_run_8_8mph_3</t>
+          <t>run 8</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.142</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.066</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Run 24 - Magnum_380_run_9_3.6mph_1</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>4.743</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1.095</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>RUN #</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>PEAKS AVG (m)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS - PEAKS AVG</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ABS AVG (m)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS ABS AVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>run 6</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.06999999999999999</v>
-      </c>
-      <c r="C2" t="inlineStr">
+        <v>0.1836666666666667</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>0.02066666666666667</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>run 7</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.1146666666666667</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>run 8</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1.712</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0.4126666666666667</v>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D9" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>

</xml_diff>

<commit_message>
added colors to cells
</commit_message>
<xml_diff>
--- a/2.12.1.345_Test Status Report.xlsx
+++ b/2.12.1.345_Test Status Report.xlsx
@@ -31,12 +31,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -57,11 +67,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -827,7 +839,7 @@
       <c r="B2" t="n">
         <v>0.036</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -835,7 +847,7 @@
       <c r="D2" t="n">
         <v>0.019</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -850,7 +862,7 @@
       <c r="B3" t="n">
         <v>0.04699999999999999</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -858,7 +870,7 @@
       <c r="D3" t="n">
         <v>0.01566666666666667</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -873,7 +885,7 @@
       <c r="B4" t="n">
         <v>0.09366666666666668</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -881,7 +893,7 @@
       <c r="D4" t="n">
         <v>0.03</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -896,7 +908,7 @@
       <c r="B5" t="n">
         <v>0.09066666666666667</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -904,7 +916,7 @@
       <c r="D5" t="n">
         <v>0.03066666666666666</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -919,7 +931,7 @@
       <c r="B6" t="n">
         <v>0.1406666666666667</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -927,7 +939,7 @@
       <c r="D6" t="n">
         <v>0.04433333333333334</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -942,7 +954,7 @@
       <c r="B7" t="n">
         <v>0.06466666666666666</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -950,7 +962,7 @@
       <c r="D7" t="n">
         <v>0.01766666666666667</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -965,7 +977,7 @@
       <c r="B8" t="n">
         <v>0.09433333333333334</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -973,7 +985,7 @@
       <c r="D8" t="n">
         <v>0.02866666666666666</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -988,7 +1000,7 @@
       <c r="B9" t="n">
         <v>0.1836666666666667</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
@@ -996,7 +1008,7 @@
       <c r="D9" t="n">
         <v>0.064</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>

</xml_diff>

<commit_message>
added stripplot only for peaks
</commit_message>
<xml_diff>
--- a/2.12.1.345_Test Status Report.xlsx
+++ b/2.12.1.345_Test Status Report.xlsx
@@ -165,6 +165,11 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -175,11 +180,11 @@
     <ext cx="34290000" cy="14287500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -193,7 +198,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -202,7 +207,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="34290000" cy="14287500"/>
+    <ext cx="28575000" cy="17145000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1091,5 +1096,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>